<commit_message>
Updating with iteration 6 candidates and results
</commit_message>
<xml_diff>
--- a/results/results_iter5.xlsx
+++ b/results/results_iter5.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danemerson/Documents/CMU/01_Research/Projects/CPA/Bayesian Optimization/cpa-bayesian-opt/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94A02C79-F888-A04B-AAF1-D1B3FC1E01DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5630C57-35EC-F441-A4FE-D1B09C114440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="18460" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="19980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -271,7 +271,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -280,6 +280,10 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -588,7 +592,7 @@
     <col min="1" max="1" width="13.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" customWidth="1"/>
+    <col min="11" max="11" width="13.6640625" style="5" customWidth="1"/>
     <col min="15" max="15" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -623,7 +627,7 @@
       <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2"/>
+      <c r="K1" s="4"/>
       <c r="L1" s="2" t="s">
         <v>50</v>
       </c>
@@ -671,7 +675,6 @@
       <c r="J2" s="3">
         <v>27.827474199983531</v>
       </c>
-      <c r="K2" s="3"/>
       <c r="L2">
         <v>30.351249094373042</v>
       </c>
@@ -721,7 +724,6 @@
       <c r="J3" s="3">
         <v>57.671753471079477</v>
       </c>
-      <c r="K3" s="3"/>
       <c r="L3">
         <v>54.694501838087326</v>
       </c>
@@ -771,7 +773,6 @@
       <c r="J4" s="3">
         <v>19.132232818680681</v>
       </c>
-      <c r="K4" s="3"/>
       <c r="L4">
         <v>31.317251187377575</v>
       </c>
@@ -821,7 +822,6 @@
       <c r="J5" s="3">
         <v>60.774089974640503</v>
       </c>
-      <c r="K5" s="3"/>
       <c r="L5">
         <v>58.075509163603201</v>
       </c>
@@ -871,7 +871,6 @@
       <c r="J6" s="3">
         <v>32.182760285552249</v>
       </c>
-      <c r="K6" s="3"/>
       <c r="L6">
         <v>16.923820001610004</v>
       </c>
@@ -921,7 +920,6 @@
       <c r="J7" s="3">
         <v>32.156293317607137</v>
       </c>
-      <c r="K7" s="3"/>
       <c r="L7">
         <v>23.106233396839031</v>
       </c>
@@ -971,7 +969,6 @@
       <c r="J8" s="3">
         <v>23.001068771456868</v>
       </c>
-      <c r="K8" s="3"/>
       <c r="L8">
         <v>28.51584511766443</v>
       </c>
@@ -1021,7 +1018,6 @@
       <c r="J9" s="3">
         <v>31.998506562105479</v>
       </c>
-      <c r="K9" s="3"/>
       <c r="L9">
         <v>16.440818955107737</v>
       </c>
@@ -1071,7 +1067,6 @@
       <c r="J10" s="3">
         <v>11.29697769717604</v>
       </c>
-      <c r="K10" s="3"/>
       <c r="L10">
         <v>1.3711863042369923</v>
       </c>
@@ -1121,7 +1116,6 @@
       <c r="J11" s="3">
         <v>51.392313326022411</v>
       </c>
-      <c r="K11" s="3"/>
       <c r="L11">
         <v>38.175866047709775</v>
       </c>
@@ -1171,7 +1165,6 @@
       <c r="J12" s="3">
         <v>101.4976113645413</v>
       </c>
-      <c r="K12" s="3"/>
       <c r="L12">
         <v>84.543966511927451</v>
       </c>
@@ -1221,7 +1214,6 @@
       <c r="J13" s="3">
         <v>101.198365920512</v>
       </c>
-      <c r="K13" s="3"/>
       <c r="L13">
         <v>80.679958139909317</v>
       </c>
@@ -1271,7 +1263,6 @@
       <c r="J14" s="3">
         <v>100.1453821526696</v>
       </c>
-      <c r="K14" s="3"/>
       <c r="L14">
         <v>80.969758767810674</v>
       </c>
@@ -1321,7 +1312,6 @@
       <c r="J15" s="3">
         <v>99.34053994917403</v>
       </c>
-      <c r="K15" s="3"/>
       <c r="L15">
         <v>82.515362116617936</v>
       </c>
@@ -1371,7 +1361,6 @@
       <c r="J16" s="3">
         <v>100.16377512827781</v>
       </c>
-      <c r="K16" s="3"/>
       <c r="L16">
         <v>90.533179488555575</v>
       </c>
@@ -1421,7 +1410,6 @@
       <c r="J17" s="3">
         <v>100.6710022913787</v>
       </c>
-      <c r="K17" s="3"/>
       <c r="L17">
         <v>86.475970697936532</v>
       </c>
@@ -1471,7 +1459,6 @@
       <c r="J18" s="3">
         <v>100.2395511827317</v>
       </c>
-      <c r="K18" s="3"/>
       <c r="L18">
         <v>84.833767139828822</v>
       </c>
@@ -1521,7 +1508,6 @@
       <c r="J19" s="3">
         <v>96.758839226135819</v>
       </c>
-      <c r="K19" s="3"/>
       <c r="L19">
         <v>83.094963372420651</v>
       </c>
@@ -1571,7 +1557,6 @@
       <c r="J20" s="3">
         <v>99.105035509204811</v>
       </c>
-      <c r="K20" s="3"/>
       <c r="L20">
         <v>80.776558349209765</v>
       </c>
@@ -1621,7 +1606,6 @@
       <c r="J21" s="3">
         <v>95.821939138937438</v>
       </c>
-      <c r="K21" s="3"/>
       <c r="L21">
         <v>78.74795395390025</v>
       </c>
@@ -1671,7 +1655,6 @@
       <c r="J22" s="3">
         <v>90.573180412358184</v>
       </c>
-      <c r="K22" s="3"/>
       <c r="L22">
         <v>76.42954893068935</v>
       </c>
@@ -1721,7 +1704,6 @@
       <c r="J23" s="3">
         <v>91.805696202405159</v>
       </c>
-      <c r="K23" s="3"/>
       <c r="L23">
         <v>82.611962325918384</v>
       </c>
@@ -1771,7 +1753,6 @@
       <c r="J24" s="3">
         <v>75.093876913484749</v>
       </c>
-      <c r="K24" s="3"/>
       <c r="L24">
         <v>82.708562535218846</v>
       </c>
@@ -1821,7 +1802,6 @@
       <c r="J25" s="3">
         <v>80.11068892484785</v>
       </c>
-      <c r="K25" s="3"/>
       <c r="L25">
         <v>89.760377814151937</v>
       </c>
@@ -1871,7 +1851,6 @@
       <c r="J26" s="3">
         <v>78.092299537586499</v>
       </c>
-      <c r="K26" s="3"/>
       <c r="L26">
         <v>70.150535326159897</v>
       </c>
@@ -1921,7 +1900,6 @@
       <c r="J27" s="3">
         <v>88.392029489581603</v>
       </c>
-      <c r="K27" s="3"/>
       <c r="L27">
         <v>95.942791209380971</v>
       </c>
@@ -1971,7 +1949,6 @@
       <c r="J28" s="3">
         <v>92.139907378254151</v>
       </c>
-      <c r="K28" s="3"/>
       <c r="L28">
         <v>90.050178442053308</v>
       </c>
@@ -2021,7 +1998,6 @@
       <c r="J29" s="3">
         <v>85.689370968014344</v>
       </c>
-      <c r="K29" s="3"/>
       <c r="L29">
         <v>86.57257090723698</v>
       </c>
@@ -2071,7 +2047,6 @@
       <c r="J30" s="3">
         <v>11.78594613529145</v>
       </c>
-      <c r="K30" s="3"/>
       <c r="L30">
         <v>17.503421257412725</v>
       </c>
@@ -2121,7 +2096,6 @@
       <c r="J31" s="3">
         <v>52.947970109739309</v>
       </c>
-      <c r="K31" s="3"/>
       <c r="L31">
         <v>53.728499745082786</v>
       </c>
@@ -2171,7 +2145,6 @@
       <c r="J32" s="3">
         <v>96.957043197859306</v>
       </c>
-      <c r="K32" s="3"/>
       <c r="L32">
         <v>92.658384093165552</v>
       </c>
@@ -2221,7 +2194,6 @@
       <c r="J33" s="3">
         <v>57.797070423445611</v>
       </c>
-      <c r="K33" s="3"/>
       <c r="L33">
         <v>57.882308745002291</v>
       </c>
@@ -2271,7 +2243,6 @@
       <c r="J34" s="3">
         <v>46.993904536879413</v>
       </c>
-      <c r="K34" s="3"/>
       <c r="L34">
         <v>25.231438001449007</v>
       </c>
@@ -2321,7 +2292,6 @@
       <c r="J35" s="3">
         <v>88.835074154890407</v>
       </c>
-      <c r="K35" s="3"/>
       <c r="L35">
         <v>78.071752488797074</v>
       </c>
@@ -2371,7 +2341,6 @@
       <c r="J36" s="3">
         <v>62.23599605778859</v>
       </c>
-      <c r="K36" s="3"/>
       <c r="L36">
         <v>23.589234443341297</v>
       </c>
@@ -2421,7 +2390,6 @@
       <c r="J37" s="3">
         <v>46.259661526325708</v>
       </c>
-      <c r="K37" s="3"/>
       <c r="L37">
         <v>52.279496605575979</v>
       </c>
@@ -2471,7 +2439,6 @@
       <c r="J38" s="3">
         <v>54.255177221828752</v>
       </c>
-      <c r="K38" s="3"/>
       <c r="L38">
         <v>36.920063326803877</v>
       </c>
@@ -2521,7 +2488,6 @@
       <c r="J39" s="3">
         <v>98.494077675121517</v>
       </c>
-      <c r="K39" s="3"/>
       <c r="L39">
         <v>97.391794348887771</v>
       </c>
@@ -2571,7 +2537,6 @@
       <c r="J40" s="3">
         <v>58.578438307810167</v>
       </c>
-      <c r="K40" s="3"/>
       <c r="L40">
         <v>20.594627955027242</v>
       </c>
@@ -2621,7 +2586,6 @@
       <c r="J41" s="3">
         <v>34.406179703671427</v>
       </c>
-      <c r="K41" s="3"/>
       <c r="L41">
         <v>56.433305605495484</v>
       </c>

</xml_diff>